<commit_message>
week 13 repo link readme added
</commit_message>
<xml_diff>
--- a/Assessments/Assessment Links.xlsx
+++ b/Assessments/Assessment Links.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Trainings\2025-Freelance\2026 01 DotNet CHD Capgemini\CU-DotNet-Jan26-B4\Assessments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{98287DCF-A704-42E7-BA76-3F5069D07DDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C626BFF8-2FCA-458C-9EBC-0211607A1FDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{3B79FAFA-49FC-4E3D-B347-76A4BB448C56}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="123">
   <si>
     <t>Sl.No</t>
   </si>
@@ -388,6 +388,21 @@
   </si>
   <si>
     <t>anjsik22/CU-DotNet-Jan26-B4</t>
+  </si>
+  <si>
+    <t>W11 - 21 Mar</t>
+  </si>
+  <si>
+    <t>W12 - 28 Mar</t>
+  </si>
+  <si>
+    <t>W13 - 04 Apr</t>
+  </si>
+  <si>
+    <t>W14 - 11 Apr</t>
+  </si>
+  <si>
+    <t>W15 - 18 Apr</t>
   </si>
 </sst>
 </file>
@@ -438,7 +453,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -448,6 +463,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC9DAF8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -525,7 +558,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -546,6 +579,15 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -863,15 +905,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B139E5B2-DFF2-4879-955D-B7DAD18F7710}">
-  <dimension ref="A1:P35"/>
+  <dimension ref="A1:U35"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="3" max="3" width="15.36328125" customWidth="1"/>
     <col min="4" max="4" width="14.7265625" customWidth="1"/>
     <col min="5" max="5" width="11" customWidth="1"/>
     <col min="6" max="6" width="12.54296875" customWidth="1"/>
+    <col min="19" max="19" width="18" customWidth="1"/>
+    <col min="21" max="21" width="8.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="53" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:21" ht="40" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -920,8 +965,23 @@
       <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q1" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" ht="44" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -950,8 +1010,13 @@
       <c r="N2" s="7"/>
       <c r="O2" s="7"/>
       <c r="P2" s="7"/>
-    </row>
-    <row r="3" spans="1:16" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q2" s="7"/>
+      <c r="R2" s="7"/>
+      <c r="S2" s="10"/>
+      <c r="T2" s="7"/>
+      <c r="U2" s="9"/>
+    </row>
+    <row r="3" spans="1:21" ht="44" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -980,8 +1045,13 @@
       <c r="N3" s="7"/>
       <c r="O3" s="7"/>
       <c r="P3" s="7"/>
-    </row>
-    <row r="4" spans="1:16" ht="73" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q3" s="7"/>
+      <c r="R3" s="7"/>
+      <c r="S3" s="10"/>
+      <c r="T3" s="7"/>
+      <c r="U3" s="9"/>
+    </row>
+    <row r="4" spans="1:21" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -1010,8 +1080,13 @@
       <c r="N4" s="7"/>
       <c r="O4" s="7"/>
       <c r="P4" s="7"/>
-    </row>
-    <row r="5" spans="1:16" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q4" s="7"/>
+      <c r="R4" s="7"/>
+      <c r="S4" s="10"/>
+      <c r="T4" s="7"/>
+      <c r="U4" s="9"/>
+    </row>
+    <row r="5" spans="1:21" ht="44" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -1030,18 +1105,23 @@
       <c r="F5" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="7"/>
-      <c r="K5" s="7"/>
-      <c r="L5" s="7"/>
-      <c r="M5" s="7"/>
-      <c r="N5" s="7"/>
-      <c r="O5" s="7"/>
-      <c r="P5" s="7"/>
-    </row>
-    <row r="6" spans="1:16" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="G5" s="8"/>
+      <c r="H5" s="8"/>
+      <c r="I5" s="8"/>
+      <c r="J5" s="8"/>
+      <c r="K5" s="8"/>
+      <c r="L5" s="8"/>
+      <c r="M5" s="8"/>
+      <c r="N5" s="8"/>
+      <c r="O5" s="8"/>
+      <c r="P5" s="8"/>
+      <c r="Q5" s="8"/>
+      <c r="R5" s="8"/>
+      <c r="S5" s="10"/>
+      <c r="T5" s="8"/>
+      <c r="U5" s="9"/>
+    </row>
+    <row r="6" spans="1:21" ht="44" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -1070,8 +1150,13 @@
       <c r="N6" s="7"/>
       <c r="O6" s="7"/>
       <c r="P6" s="7"/>
-    </row>
-    <row r="7" spans="1:16" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q6" s="7"/>
+      <c r="R6" s="7"/>
+      <c r="S6" s="10"/>
+      <c r="T6" s="7"/>
+      <c r="U6" s="9"/>
+    </row>
+    <row r="7" spans="1:21" ht="44" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -1100,8 +1185,13 @@
       <c r="N7" s="7"/>
       <c r="O7" s="7"/>
       <c r="P7" s="7"/>
-    </row>
-    <row r="8" spans="1:16" ht="73" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q7" s="7"/>
+      <c r="R7" s="7"/>
+      <c r="S7" s="10"/>
+      <c r="T7" s="7"/>
+      <c r="U7" s="9"/>
+    </row>
+    <row r="8" spans="1:21" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -1130,8 +1220,13 @@
       <c r="N8" s="7"/>
       <c r="O8" s="7"/>
       <c r="P8" s="7"/>
-    </row>
-    <row r="9" spans="1:16" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q8" s="7"/>
+      <c r="R8" s="7"/>
+      <c r="S8" s="10"/>
+      <c r="T8" s="7"/>
+      <c r="U8" s="9"/>
+    </row>
+    <row r="9" spans="1:21" ht="44" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -1150,18 +1245,23 @@
       <c r="F9" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
-      <c r="J9" s="7"/>
-      <c r="K9" s="7"/>
-      <c r="L9" s="7"/>
-      <c r="M9" s="7"/>
-      <c r="N9" s="7"/>
-      <c r="O9" s="7"/>
-      <c r="P9" s="7"/>
-    </row>
-    <row r="10" spans="1:16" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="8"/>
+      <c r="O9" s="8"/>
+      <c r="P9" s="8"/>
+      <c r="Q9" s="8"/>
+      <c r="R9" s="8"/>
+      <c r="S9" s="10"/>
+      <c r="T9" s="8"/>
+      <c r="U9" s="9"/>
+    </row>
+    <row r="10" spans="1:21" ht="44" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -1190,8 +1290,13 @@
       <c r="N10" s="7"/>
       <c r="O10" s="7"/>
       <c r="P10" s="7"/>
-    </row>
-    <row r="11" spans="1:16" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q10" s="7"/>
+      <c r="R10" s="7"/>
+      <c r="S10" s="10"/>
+      <c r="T10" s="7"/>
+      <c r="U10" s="9"/>
+    </row>
+    <row r="11" spans="1:21" ht="44" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -1220,8 +1325,13 @@
       <c r="N11" s="7"/>
       <c r="O11" s="7"/>
       <c r="P11" s="7"/>
-    </row>
-    <row r="12" spans="1:16" ht="131" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q11" s="7"/>
+      <c r="R11" s="7"/>
+      <c r="S11" s="10"/>
+      <c r="T11" s="7"/>
+      <c r="U11" s="9"/>
+    </row>
+    <row r="12" spans="1:21" ht="73" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -1250,8 +1360,13 @@
       <c r="N12" s="7"/>
       <c r="O12" s="7"/>
       <c r="P12" s="7"/>
-    </row>
-    <row r="13" spans="1:16" ht="131" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q12" s="7"/>
+      <c r="R12" s="7"/>
+      <c r="S12" s="10"/>
+      <c r="T12" s="7"/>
+      <c r="U12" s="9"/>
+    </row>
+    <row r="13" spans="1:21" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -1280,8 +1395,13 @@
       <c r="N13" s="7"/>
       <c r="O13" s="7"/>
       <c r="P13" s="7"/>
-    </row>
-    <row r="14" spans="1:16" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q13" s="7"/>
+      <c r="R13" s="7"/>
+      <c r="S13" s="10"/>
+      <c r="T13" s="7"/>
+      <c r="U13" s="9"/>
+    </row>
+    <row r="14" spans="1:21" ht="44" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -1310,8 +1430,13 @@
       <c r="N14" s="7"/>
       <c r="O14" s="7"/>
       <c r="P14" s="7"/>
-    </row>
-    <row r="15" spans="1:16" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q14" s="7"/>
+      <c r="R14" s="7"/>
+      <c r="S14" s="10"/>
+      <c r="T14" s="7"/>
+      <c r="U14" s="9"/>
+    </row>
+    <row r="15" spans="1:21" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -1340,8 +1465,13 @@
       <c r="N15" s="7"/>
       <c r="O15" s="7"/>
       <c r="P15" s="7"/>
-    </row>
-    <row r="16" spans="1:16" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q15" s="7"/>
+      <c r="R15" s="7"/>
+      <c r="S15" s="10"/>
+      <c r="T15" s="7"/>
+      <c r="U15" s="9"/>
+    </row>
+    <row r="16" spans="1:21" ht="44" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -1370,8 +1500,13 @@
       <c r="N16" s="7"/>
       <c r="O16" s="7"/>
       <c r="P16" s="7"/>
-    </row>
-    <row r="17" spans="1:16" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q16" s="7"/>
+      <c r="R16" s="7"/>
+      <c r="S16" s="10"/>
+      <c r="T16" s="7"/>
+      <c r="U16" s="9"/>
+    </row>
+    <row r="17" spans="1:21" ht="44" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -1400,8 +1535,13 @@
       <c r="N17" s="7"/>
       <c r="O17" s="7"/>
       <c r="P17" s="7"/>
-    </row>
-    <row r="18" spans="1:16" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q17" s="7"/>
+      <c r="R17" s="7"/>
+      <c r="S17" s="10"/>
+      <c r="T17" s="7"/>
+      <c r="U17" s="9"/>
+    </row>
+    <row r="18" spans="1:21" ht="44" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -1430,8 +1570,13 @@
       <c r="N18" s="7"/>
       <c r="O18" s="7"/>
       <c r="P18" s="7"/>
-    </row>
-    <row r="19" spans="1:16" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q18" s="7"/>
+      <c r="R18" s="7"/>
+      <c r="S18" s="10"/>
+      <c r="T18" s="7"/>
+      <c r="U18" s="9"/>
+    </row>
+    <row r="19" spans="1:21" ht="44" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -1460,8 +1605,13 @@
       <c r="N19" s="7"/>
       <c r="O19" s="7"/>
       <c r="P19" s="7"/>
-    </row>
-    <row r="20" spans="1:16" ht="102" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q19" s="7"/>
+      <c r="R19" s="7"/>
+      <c r="S19" s="10"/>
+      <c r="T19" s="7"/>
+      <c r="U19" s="9"/>
+    </row>
+    <row r="20" spans="1:21" ht="73" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -1490,8 +1640,13 @@
       <c r="N20" s="7"/>
       <c r="O20" s="7"/>
       <c r="P20" s="7"/>
-    </row>
-    <row r="21" spans="1:16" ht="73" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q20" s="7"/>
+      <c r="R20" s="7"/>
+      <c r="S20" s="10"/>
+      <c r="T20" s="7"/>
+      <c r="U20" s="9"/>
+    </row>
+    <row r="21" spans="1:21" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -1520,8 +1675,13 @@
       <c r="N21" s="7"/>
       <c r="O21" s="7"/>
       <c r="P21" s="7"/>
-    </row>
-    <row r="22" spans="1:16" ht="145.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q21" s="7"/>
+      <c r="R21" s="7"/>
+      <c r="S21" s="10"/>
+      <c r="T21" s="7"/>
+      <c r="U21" s="9"/>
+    </row>
+    <row r="22" spans="1:21" ht="102" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -1550,8 +1710,13 @@
       <c r="N22" s="7"/>
       <c r="O22" s="7"/>
       <c r="P22" s="7"/>
-    </row>
-    <row r="23" spans="1:16" ht="145.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q22" s="7"/>
+      <c r="R22" s="7"/>
+      <c r="S22" s="10"/>
+      <c r="T22" s="7"/>
+      <c r="U22" s="9"/>
+    </row>
+    <row r="23" spans="1:21" ht="102" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -1580,8 +1745,13 @@
       <c r="N23" s="7"/>
       <c r="O23" s="7"/>
       <c r="P23" s="7"/>
-    </row>
-    <row r="24" spans="1:16" ht="73" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q23" s="7"/>
+      <c r="R23" s="7"/>
+      <c r="S23" s="10"/>
+      <c r="T23" s="7"/>
+      <c r="U23" s="9"/>
+    </row>
+    <row r="24" spans="1:21" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A24" s="3">
         <v>23</v>
       </c>
@@ -1610,8 +1780,13 @@
       <c r="N24" s="7"/>
       <c r="O24" s="7"/>
       <c r="P24" s="7"/>
-    </row>
-    <row r="25" spans="1:16" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q24" s="7"/>
+      <c r="R24" s="7"/>
+      <c r="S24" s="10"/>
+      <c r="T24" s="7"/>
+      <c r="U24" s="9"/>
+    </row>
+    <row r="25" spans="1:21" ht="44" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A25" s="3">
         <v>24</v>
       </c>
@@ -1640,8 +1815,13 @@
       <c r="N25" s="7"/>
       <c r="O25" s="7"/>
       <c r="P25" s="7"/>
-    </row>
-    <row r="26" spans="1:16" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q25" s="7"/>
+      <c r="R25" s="7"/>
+      <c r="S25" s="10"/>
+      <c r="T25" s="7"/>
+      <c r="U25" s="9"/>
+    </row>
+    <row r="26" spans="1:21" ht="44" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A26" s="3">
         <v>25</v>
       </c>
@@ -1670,8 +1850,13 @@
       <c r="N26" s="7"/>
       <c r="O26" s="7"/>
       <c r="P26" s="7"/>
-    </row>
-    <row r="27" spans="1:16" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q26" s="7"/>
+      <c r="R26" s="7"/>
+      <c r="S26" s="10"/>
+      <c r="T26" s="7"/>
+      <c r="U26" s="9"/>
+    </row>
+    <row r="27" spans="1:21" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A27" s="3">
         <v>26</v>
       </c>
@@ -1700,8 +1885,13 @@
       <c r="N27" s="7"/>
       <c r="O27" s="7"/>
       <c r="P27" s="7"/>
-    </row>
-    <row r="28" spans="1:16" ht="102" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q27" s="7"/>
+      <c r="R27" s="7"/>
+      <c r="S27" s="10"/>
+      <c r="T27" s="7"/>
+      <c r="U27" s="9"/>
+    </row>
+    <row r="28" spans="1:21" ht="73" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="3">
         <v>27</v>
       </c>
@@ -1730,8 +1920,13 @@
       <c r="N28" s="7"/>
       <c r="O28" s="7"/>
       <c r="P28" s="7"/>
-    </row>
-    <row r="29" spans="1:16" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q28" s="7"/>
+      <c r="R28" s="7"/>
+      <c r="S28" s="10"/>
+      <c r="T28" s="7"/>
+      <c r="U28" s="9"/>
+    </row>
+    <row r="29" spans="1:21" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A29" s="3">
         <v>28</v>
       </c>
@@ -1760,8 +1955,13 @@
       <c r="N29" s="7"/>
       <c r="O29" s="7"/>
       <c r="P29" s="7"/>
-    </row>
-    <row r="30" spans="1:16" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q29" s="7"/>
+      <c r="R29" s="7"/>
+      <c r="S29" s="10"/>
+      <c r="T29" s="7"/>
+      <c r="U29" s="9"/>
+    </row>
+    <row r="30" spans="1:21" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A30" s="3">
         <v>29</v>
       </c>
@@ -1790,8 +1990,13 @@
       <c r="N30" s="7"/>
       <c r="O30" s="7"/>
       <c r="P30" s="7"/>
-    </row>
-    <row r="31" spans="1:16" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q30" s="7"/>
+      <c r="R30" s="7"/>
+      <c r="S30" s="10"/>
+      <c r="T30" s="7"/>
+      <c r="U30" s="9"/>
+    </row>
+    <row r="31" spans="1:21" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A31" s="3">
         <v>30</v>
       </c>
@@ -1820,8 +2025,13 @@
       <c r="N31" s="7"/>
       <c r="O31" s="7"/>
       <c r="P31" s="7"/>
-    </row>
-    <row r="32" spans="1:16" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q31" s="7"/>
+      <c r="R31" s="7"/>
+      <c r="S31" s="10"/>
+      <c r="T31" s="7"/>
+      <c r="U31" s="9"/>
+    </row>
+    <row r="32" spans="1:21" ht="44" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A32" s="3">
         <v>31</v>
       </c>
@@ -1850,8 +2060,13 @@
       <c r="N32" s="7"/>
       <c r="O32" s="7"/>
       <c r="P32" s="7"/>
-    </row>
-    <row r="33" spans="1:16" ht="73" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q32" s="7"/>
+      <c r="R32" s="7"/>
+      <c r="S32" s="10"/>
+      <c r="T32" s="7"/>
+      <c r="U32" s="9"/>
+    </row>
+    <row r="33" spans="1:21" ht="44" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A33" s="3">
         <v>32</v>
       </c>
@@ -1880,8 +2095,13 @@
       <c r="N33" s="7"/>
       <c r="O33" s="7"/>
       <c r="P33" s="7"/>
-    </row>
-    <row r="34" spans="1:16" ht="73" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q33" s="7"/>
+      <c r="R33" s="7"/>
+      <c r="S33" s="10"/>
+      <c r="T33" s="7"/>
+      <c r="U33" s="9"/>
+    </row>
+    <row r="34" spans="1:21" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A34" s="3">
         <v>33</v>
       </c>
@@ -1910,8 +2130,13 @@
       <c r="N34" s="7"/>
       <c r="O34" s="7"/>
       <c r="P34" s="7"/>
-    </row>
-    <row r="35" spans="1:16" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q34" s="7"/>
+      <c r="R34" s="7"/>
+      <c r="S34" s="10"/>
+      <c r="T34" s="7"/>
+      <c r="U34" s="9"/>
+    </row>
+    <row r="35" spans="1:21" ht="44" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A35" s="3">
         <v>34</v>
       </c>
@@ -1940,6 +2165,11 @@
       <c r="N35" s="7"/>
       <c r="O35" s="7"/>
       <c r="P35" s="7"/>
+      <c r="Q35" s="7"/>
+      <c r="R35" s="7"/>
+      <c r="S35" s="10"/>
+      <c r="T35" s="7"/>
+      <c r="U35" s="9"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>